<commit_message>
update Django.xlsx with new content
</commit_message>
<xml_diff>
--- a/Django.xlsx
+++ b/Django.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Django\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8498F0FF-D04C-4621-94EB-CE0A7202299C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AFEA7D-8474-4B57-87E1-5A580D0A72A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0FFEE4F1-0908-4232-AD41-10A73D286687}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="72">
   <si>
     <t>Let's separate the whole Django into two part, backend and api</t>
   </si>
@@ -241,6 +241,66 @@
   </si>
   <si>
     <t>venv\Scripts\activate</t>
+  </si>
+  <si>
+    <t>import uuid</t>
+  </si>
+  <si>
+    <t>class Product(models.Model):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    id = models.UUIDField(</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        primary_key=True,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        default=uuid.uuid4,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        editable=False</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This will create a uuid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">        raise PermissionDenied("You do not have permission.")</t>
+  </si>
+  <si>
+    <t>from rest_framework import viewsets</t>
+  </si>
+  <si>
+    <t>from rest_framework.permissions import IsAuthenticated, AllowAny</t>
+  </si>
+  <si>
+    <t>from rest_framework.exceptions import PermissionDenied</t>
+  </si>
+  <si>
+    <t>class PostViewSet(viewsets.ModelViewSet):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    queryset = Post.objects.all()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    serializer_class = PostSerializer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    def get_permissions(self):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        # Allow only list page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        if self.action == "list":</t>
+  </si>
+  <si>
+    <t xml:space="preserve">            return [IsAuthenticated()]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        # Block details/update/delete/create</t>
   </si>
 </sst>
 </file>
@@ -654,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D723068F-9FA8-4FF8-81EB-8C964E855B9A}">
-  <dimension ref="B3:E44"/>
+  <dimension ref="B3:E83"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="70.90625" customWidth="1"/>
@@ -895,6 +955,106 @@
         <v>42</v>
       </c>
     </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B52" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B53" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B54" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B55" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B56" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B57" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B59" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B68" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B69" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B70" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B72" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B73" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B74" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B76" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B78" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B79" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B80" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B82" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B83" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>